<commit_message>
new updates on the panel board
</commit_message>
<xml_diff>
--- a/public/Grading_Template.xlsx
+++ b/public/Grading_Template.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Justine\solar-converter\public\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{20383263-86C6-4382-AF0B-F2CCBE2EAFE9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DE88B0D8-8F1D-426E-95FE-94B839C8E055}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{4EF88AD7-D076-41CD-BCFA-A05F6A55A005}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="1" xr2:uid="{4EF88AD7-D076-41CD-BCFA-A05F6A55A005}"/>
   </bookViews>
   <sheets>
     <sheet name="GROUPGRADE" sheetId="1" r:id="rId1"/>
@@ -1214,58 +1214,25 @@
     <xf numFmtId="0" fontId="34" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1280,39 +1247,44 @@
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="31" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="31" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="32" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="34" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1323,6 +1295,34 @@
     <xf numFmtId="0" fontId="35" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1338,6 +1338,154 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>172827</xdr:colOff>
+      <xdr:row>56</xdr:row>
+      <xdr:rowOff>2</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>864125</xdr:colOff>
+      <xdr:row>57</xdr:row>
+      <xdr:rowOff>172634</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="6" name="Picture 5">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{049E1B46-64DE-4B68-316D-EF0FC41346C1}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1">
+          <a:extLst>
+            <a:ext uri="{BEBA8EAE-BF5A-486C-A8C5-ECC9F3942E4B}">
+              <a14:imgProps xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+                <a14:imgLayer r:embed="rId2">
+                  <a14:imgEffect>
+                    <a14:backgroundRemoval t="9559" b="89706" l="6707" r="89634">
+                      <a14:foregroundMark x1="17073" y1="85294" x2="38415" y2="68382"/>
+                      <a14:foregroundMark x1="27439" y1="65441" x2="68293" y2="49265"/>
+                      <a14:foregroundMark x1="20732" y1="49265" x2="31707" y2="50735"/>
+                      <a14:foregroundMark x1="6707" y1="80882" x2="18293" y2="74265"/>
+                      <a14:foregroundMark x1="62195" y1="55147" x2="86585" y2="35294"/>
+                      <a14:foregroundMark x1="53659" y1="36765" x2="53659" y2="36765"/>
+                      <a14:foregroundMark x1="39634" y1="36765" x2="39634" y2="36765"/>
+                      <a14:foregroundMark x1="39634" y1="46324" x2="39634" y2="46324"/>
+                      <a14:foregroundMark x1="47561" y1="36765" x2="47561" y2="36765"/>
+                    </a14:backgroundRemoval>
+                  </a14:imgEffect>
+                </a14:imgLayer>
+              </a14:imgProps>
+            </a:ext>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="3542909" y="23755548"/>
+          <a:ext cx="691298" cy="573272"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>304800</xdr:colOff>
+      <xdr:row>27</xdr:row>
+      <xdr:rowOff>228601</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>321184</xdr:colOff>
+      <xdr:row>29</xdr:row>
+      <xdr:rowOff>181387</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="Picture 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{819F39E2-4AB0-4185-9D0D-384B9A3D875F}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1">
+          <a:extLst>
+            <a:ext uri="{BEBA8EAE-BF5A-486C-A8C5-ECC9F3942E4B}">
+              <a14:imgProps xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+                <a14:imgLayer r:embed="rId2">
+                  <a14:imgEffect>
+                    <a14:backgroundRemoval t="9559" b="89706" l="6707" r="89634">
+                      <a14:foregroundMark x1="17073" y1="85294" x2="38415" y2="68382"/>
+                      <a14:foregroundMark x1="27439" y1="65441" x2="68293" y2="49265"/>
+                      <a14:foregroundMark x1="20732" y1="49265" x2="31707" y2="50735"/>
+                      <a14:foregroundMark x1="6707" y1="80882" x2="18293" y2="74265"/>
+                      <a14:foregroundMark x1="62195" y1="55147" x2="86585" y2="35294"/>
+                      <a14:foregroundMark x1="53659" y1="36765" x2="53659" y2="36765"/>
+                      <a14:foregroundMark x1="39634" y1="36765" x2="39634" y2="36765"/>
+                      <a14:foregroundMark x1="39634" y1="46324" x2="39634" y2="46324"/>
+                      <a14:foregroundMark x1="47561" y1="36765" x2="47561" y2="36765"/>
+                    </a14:backgroundRemoval>
+                  </a14:imgEffect>
+                </a14:imgLayer>
+              </a14:imgProps>
+            </a:ext>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="7434943" y="7130144"/>
+          <a:ext cx="691298" cy="573272"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1650,7 +1798,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="25.8" x14ac:dyDescent="0.5">
-      <c r="A1" s="56" t="s">
+      <c r="A1" s="72" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="57"/>
@@ -1661,7 +1809,7 @@
       <c r="G1" s="57"/>
     </row>
     <row r="2" spans="1:7" ht="17.399999999999999" x14ac:dyDescent="0.35">
-      <c r="A2" s="58" t="s">
+      <c r="A2" s="73" t="s">
         <v>1</v>
       </c>
       <c r="B2" s="57"/>
@@ -1681,120 +1829,120 @@
       <c r="G3" s="2"/>
     </row>
     <row r="4" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A4" s="59" t="s">
+      <c r="A4" s="74" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="54"/>
-      <c r="C4" s="54"/>
-      <c r="D4" s="54"/>
-      <c r="E4" s="54"/>
-      <c r="F4" s="54"/>
-      <c r="G4" s="55"/>
+      <c r="B4" s="75"/>
+      <c r="C4" s="75"/>
+      <c r="D4" s="75"/>
+      <c r="E4" s="75"/>
+      <c r="F4" s="75"/>
+      <c r="G4" s="76"/>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A5" s="60" t="s">
+      <c r="A5" s="80" t="s">
         <v>3</v>
       </c>
-      <c r="B5" s="61"/>
-      <c r="C5" s="61"/>
-      <c r="D5" s="61"/>
-      <c r="E5" s="61"/>
-      <c r="F5" s="61"/>
-      <c r="G5" s="62"/>
+      <c r="B5" s="64"/>
+      <c r="C5" s="64"/>
+      <c r="D5" s="64"/>
+      <c r="E5" s="64"/>
+      <c r="F5" s="64"/>
+      <c r="G5" s="65"/>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A6" s="63"/>
+      <c r="A6" s="81"/>
       <c r="B6" s="57"/>
       <c r="C6" s="57"/>
       <c r="D6" s="57"/>
       <c r="E6" s="57"/>
       <c r="F6" s="57"/>
-      <c r="G6" s="64"/>
+      <c r="G6" s="58"/>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A7" s="65"/>
+      <c r="A7" s="59"/>
       <c r="B7" s="57"/>
       <c r="C7" s="57"/>
       <c r="D7" s="57"/>
       <c r="E7" s="57"/>
       <c r="F7" s="57"/>
-      <c r="G7" s="64"/>
+      <c r="G7" s="58"/>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A8" s="53" t="s">
+      <c r="A8" s="86" t="s">
         <v>4</v>
       </c>
-      <c r="B8" s="54"/>
-      <c r="C8" s="54"/>
-      <c r="D8" s="54"/>
-      <c r="E8" s="54"/>
-      <c r="F8" s="54"/>
-      <c r="G8" s="55"/>
+      <c r="B8" s="75"/>
+      <c r="C8" s="75"/>
+      <c r="D8" s="75"/>
+      <c r="E8" s="75"/>
+      <c r="F8" s="75"/>
+      <c r="G8" s="76"/>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A9" s="67"/>
-      <c r="B9" s="54"/>
-      <c r="C9" s="54"/>
-      <c r="D9" s="54"/>
-      <c r="E9" s="54"/>
-      <c r="F9" s="54"/>
-      <c r="G9" s="55"/>
+      <c r="A9" s="79"/>
+      <c r="B9" s="75"/>
+      <c r="C9" s="75"/>
+      <c r="D9" s="75"/>
+      <c r="E9" s="75"/>
+      <c r="F9" s="75"/>
+      <c r="G9" s="76"/>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A10" s="65"/>
+      <c r="A10" s="59"/>
       <c r="B10" s="57"/>
       <c r="C10" s="57"/>
       <c r="D10" s="57"/>
       <c r="E10" s="57"/>
       <c r="F10" s="57"/>
-      <c r="G10" s="64"/>
+      <c r="G10" s="58"/>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A11" s="65"/>
+      <c r="A11" s="59"/>
       <c r="B11" s="57"/>
       <c r="C11" s="57"/>
       <c r="D11" s="57"/>
       <c r="E11" s="57"/>
       <c r="F11" s="57"/>
-      <c r="G11" s="64"/>
+      <c r="G11" s="58"/>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A12" s="68"/>
-      <c r="B12" s="69"/>
-      <c r="C12" s="69"/>
-      <c r="D12" s="69"/>
-      <c r="E12" s="69"/>
-      <c r="F12" s="69"/>
-      <c r="G12" s="70"/>
+      <c r="A12" s="60"/>
+      <c r="B12" s="54"/>
+      <c r="C12" s="54"/>
+      <c r="D12" s="54"/>
+      <c r="E12" s="54"/>
+      <c r="F12" s="54"/>
+      <c r="G12" s="55"/>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A13" s="60" t="s">
+      <c r="A13" s="80" t="s">
         <v>5</v>
       </c>
-      <c r="B13" s="61"/>
-      <c r="C13" s="61"/>
-      <c r="D13" s="61"/>
-      <c r="E13" s="61"/>
-      <c r="F13" s="61"/>
-      <c r="G13" s="62"/>
+      <c r="B13" s="64"/>
+      <c r="C13" s="64"/>
+      <c r="D13" s="64"/>
+      <c r="E13" s="64"/>
+      <c r="F13" s="64"/>
+      <c r="G13" s="65"/>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A14" s="63"/>
+      <c r="A14" s="81"/>
       <c r="B14" s="57"/>
       <c r="C14" s="57"/>
       <c r="D14" s="57"/>
       <c r="E14" s="57"/>
       <c r="F14" s="57"/>
-      <c r="G14" s="64"/>
+      <c r="G14" s="58"/>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A15" s="68"/>
-      <c r="B15" s="69"/>
-      <c r="C15" s="69"/>
-      <c r="D15" s="69"/>
-      <c r="E15" s="69"/>
-      <c r="F15" s="69"/>
-      <c r="G15" s="70"/>
+      <c r="A15" s="60"/>
+      <c r="B15" s="54"/>
+      <c r="C15" s="54"/>
+      <c r="D15" s="54"/>
+      <c r="E15" s="54"/>
+      <c r="F15" s="54"/>
+      <c r="G15" s="55"/>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A16" s="2"/>
@@ -1806,41 +1954,41 @@
       <c r="G16" s="2"/>
     </row>
     <row r="17" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A17" s="71" t="s">
+      <c r="A17" s="82" t="s">
         <v>6</v>
       </c>
-      <c r="B17" s="61"/>
-      <c r="C17" s="61"/>
-      <c r="D17" s="61"/>
-      <c r="E17" s="61"/>
-      <c r="F17" s="61"/>
-      <c r="G17" s="62"/>
+      <c r="B17" s="64"/>
+      <c r="C17" s="64"/>
+      <c r="D17" s="64"/>
+      <c r="E17" s="64"/>
+      <c r="F17" s="64"/>
+      <c r="G17" s="65"/>
     </row>
     <row r="18" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A18" s="72">
+      <c r="A18" s="83">
         <v>1</v>
       </c>
-      <c r="B18" s="61"/>
-      <c r="C18" s="61"/>
-      <c r="D18" s="62"/>
-      <c r="E18" s="72">
+      <c r="B18" s="64"/>
+      <c r="C18" s="64"/>
+      <c r="D18" s="65"/>
+      <c r="E18" s="83">
         <v>3</v>
       </c>
-      <c r="F18" s="61"/>
-      <c r="G18" s="62"/>
+      <c r="F18" s="64"/>
+      <c r="G18" s="65"/>
     </row>
     <row r="19" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A19" s="72">
+      <c r="A19" s="83">
         <v>2</v>
       </c>
-      <c r="B19" s="61"/>
-      <c r="C19" s="61"/>
-      <c r="D19" s="62"/>
-      <c r="E19" s="73">
+      <c r="B19" s="64"/>
+      <c r="C19" s="64"/>
+      <c r="D19" s="65"/>
+      <c r="E19" s="84">
         <v>4</v>
       </c>
-      <c r="F19" s="61"/>
-      <c r="G19" s="62"/>
+      <c r="F19" s="64"/>
+      <c r="G19" s="65"/>
     </row>
     <row r="20" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A20" s="3"/>
@@ -1861,57 +2009,57 @@
       <c r="G21" s="2"/>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A22" s="74" t="s">
+      <c r="A22" s="85" t="s">
         <v>7</v>
       </c>
-      <c r="B22" s="61"/>
-      <c r="C22" s="61"/>
-      <c r="D22" s="61"/>
-      <c r="E22" s="61"/>
-      <c r="F22" s="61"/>
-      <c r="G22" s="62"/>
+      <c r="B22" s="64"/>
+      <c r="C22" s="64"/>
+      <c r="D22" s="64"/>
+      <c r="E22" s="64"/>
+      <c r="F22" s="64"/>
+      <c r="G22" s="65"/>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A23" s="66" t="s">
+      <c r="A23" s="78" t="s">
         <v>8</v>
       </c>
-      <c r="B23" s="61"/>
-      <c r="C23" s="61"/>
-      <c r="D23" s="61"/>
-      <c r="E23" s="66" t="s">
+      <c r="B23" s="64"/>
+      <c r="C23" s="64"/>
+      <c r="D23" s="64"/>
+      <c r="E23" s="78" t="s">
         <v>9</v>
       </c>
-      <c r="F23" s="62"/>
+      <c r="F23" s="65"/>
       <c r="G23" s="4" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A24" s="66" t="s">
+      <c r="A24" s="78" t="s">
         <v>11</v>
       </c>
-      <c r="B24" s="61"/>
-      <c r="C24" s="61"/>
-      <c r="D24" s="61"/>
-      <c r="E24" s="61"/>
-      <c r="F24" s="61"/>
+      <c r="B24" s="64"/>
+      <c r="C24" s="64"/>
+      <c r="D24" s="64"/>
+      <c r="E24" s="64"/>
+      <c r="F24" s="64"/>
       <c r="G24" s="4" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="25" spans="1:7" ht="30" x14ac:dyDescent="0.5">
-      <c r="A25" s="76">
+      <c r="A25" s="63">
         <f>SUM(G31:G36)+SUM(G40:G41)+SUM(G45:G47)</f>
         <v>0</v>
       </c>
-      <c r="B25" s="61"/>
-      <c r="C25" s="61"/>
-      <c r="D25" s="62"/>
-      <c r="E25" s="76">
+      <c r="B25" s="64"/>
+      <c r="C25" s="64"/>
+      <c r="D25" s="65"/>
+      <c r="E25" s="63">
         <f>SUM(G53:G56)</f>
         <v>0</v>
       </c>
-      <c r="F25" s="62"/>
+      <c r="F25" s="65"/>
       <c r="G25" s="5">
         <f>SUM(G31:G36)+SUM(G40:G41)+SUM(G45:G47)+SUM(G53:G56)</f>
         <v>0</v>
@@ -1927,7 +2075,7 @@
       <c r="G26" s="6"/>
     </row>
     <row r="27" spans="1:7" ht="19.8" x14ac:dyDescent="0.4">
-      <c r="A27" s="77" t="s">
+      <c r="A27" s="66" t="s">
         <v>13</v>
       </c>
       <c r="B27" s="57"/>
@@ -1980,7 +2128,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="31" spans="1:7" ht="60" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:7" ht="36" x14ac:dyDescent="0.3">
       <c r="A31" s="14" t="s">
         <v>22</v>
       </c>
@@ -2001,7 +2149,7 @@
       </c>
       <c r="G31" s="16"/>
     </row>
-    <row r="32" spans="1:7" ht="108" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:7" ht="60" x14ac:dyDescent="0.3">
       <c r="A32" s="14" t="s">
         <v>28</v>
       </c>
@@ -2022,7 +2170,7 @@
       </c>
       <c r="G32" s="16"/>
     </row>
-    <row r="33" spans="1:7" ht="300" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:7" ht="168" x14ac:dyDescent="0.3">
       <c r="A33" s="14" t="s">
         <v>34</v>
       </c>
@@ -2043,7 +2191,7 @@
       </c>
       <c r="G33" s="16"/>
     </row>
-    <row r="34" spans="1:7" ht="84" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:7" ht="72" x14ac:dyDescent="0.3">
       <c r="A34" s="17" t="s">
         <v>40</v>
       </c>
@@ -2064,7 +2212,7 @@
       </c>
       <c r="G34" s="16"/>
     </row>
-    <row r="35" spans="1:7" ht="132" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:7" ht="120" x14ac:dyDescent="0.3">
       <c r="A35" s="17" t="s">
         <v>46</v>
       </c>
@@ -2085,7 +2233,7 @@
       </c>
       <c r="G35" s="16"/>
     </row>
-    <row r="36" spans="1:7" ht="108" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:7" ht="96" x14ac:dyDescent="0.3">
       <c r="A36" s="17" t="s">
         <v>52</v>
       </c>
@@ -2149,7 +2297,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="40" spans="1:7" ht="156" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:7" ht="120" x14ac:dyDescent="0.3">
       <c r="A40" s="26" t="s">
         <v>61</v>
       </c>
@@ -2201,14 +2349,14 @@
       <c r="G42" s="29"/>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A43" s="78" t="s">
+      <c r="A43" s="67" t="s">
         <v>73</v>
       </c>
-      <c r="B43" s="79"/>
-      <c r="C43" s="79"/>
-      <c r="D43" s="79"/>
-      <c r="E43" s="79"/>
-      <c r="F43" s="80"/>
+      <c r="B43" s="68"/>
+      <c r="C43" s="68"/>
+      <c r="D43" s="68"/>
+      <c r="E43" s="68"/>
+      <c r="F43" s="69"/>
       <c r="G43" s="30"/>
     </row>
     <row r="44" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
@@ -2316,7 +2464,7 @@
       <c r="G49" s="29"/>
     </row>
     <row r="50" spans="1:7" ht="19.8" x14ac:dyDescent="0.4">
-      <c r="A50" s="77" t="s">
+      <c r="A50" s="66" t="s">
         <v>92</v>
       </c>
       <c r="B50" s="57"/>
@@ -2335,7 +2483,7 @@
       <c r="F51" s="36"/>
       <c r="G51" s="35"/>
     </row>
-    <row r="52" spans="1:7" ht="72" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:7" ht="54" x14ac:dyDescent="0.3">
       <c r="A52" s="37" t="s">
         <v>15</v>
       </c>
@@ -2358,7 +2506,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="53" spans="1:7" ht="72" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:7" ht="60" x14ac:dyDescent="0.3">
       <c r="A53" s="40" t="s">
         <v>93</v>
       </c>
@@ -2379,7 +2527,7 @@
       </c>
       <c r="G53" s="16"/>
     </row>
-    <row r="54" spans="1:7" ht="72" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:7" ht="60" x14ac:dyDescent="0.3">
       <c r="A54" s="40" t="s">
         <v>99</v>
       </c>
@@ -2400,7 +2548,7 @@
       </c>
       <c r="G54" s="16"/>
     </row>
-    <row r="55" spans="1:7" ht="72" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:7" ht="60" x14ac:dyDescent="0.3">
       <c r="A55" s="42" t="s">
         <v>105</v>
       </c>
@@ -2453,24 +2601,24 @@
     </row>
     <row r="58" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A58" s="2"/>
-      <c r="B58" s="81" t="s">
+      <c r="B58" s="70" t="s">
         <v>117</v>
       </c>
-      <c r="C58" s="81"/>
-      <c r="D58" s="81"/>
-      <c r="E58" s="81"/>
-      <c r="F58" s="81"/>
+      <c r="C58" s="70"/>
+      <c r="D58" s="70"/>
+      <c r="E58" s="70"/>
+      <c r="F58" s="70"/>
       <c r="G58" s="2"/>
     </row>
     <row r="59" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A59" s="2"/>
-      <c r="B59" s="82" t="s">
+      <c r="B59" s="71" t="s">
         <v>118</v>
       </c>
-      <c r="C59" s="82"/>
-      <c r="D59" s="82"/>
-      <c r="E59" s="82"/>
-      <c r="F59" s="82"/>
+      <c r="C59" s="71"/>
+      <c r="D59" s="71"/>
+      <c r="E59" s="71"/>
+      <c r="F59" s="71"/>
       <c r="G59" s="2"/>
     </row>
     <row r="60" spans="1:7" x14ac:dyDescent="0.3">
@@ -2492,7 +2640,7 @@
       <c r="G61" s="2"/>
     </row>
     <row r="62" spans="1:7" ht="25.8" x14ac:dyDescent="0.5">
-      <c r="A62" s="56" t="s">
+      <c r="A62" s="72" t="s">
         <v>119</v>
       </c>
       <c r="B62" s="57"/>
@@ -2503,7 +2651,7 @@
       <c r="G62" s="57"/>
     </row>
     <row r="63" spans="1:7" ht="17.399999999999999" x14ac:dyDescent="0.35">
-      <c r="A63" s="58" t="s">
+      <c r="A63" s="73" t="s">
         <v>1</v>
       </c>
       <c r="B63" s="57"/>
@@ -2523,120 +2671,120 @@
       <c r="G64" s="2"/>
     </row>
     <row r="65" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A65" s="59" t="s">
+      <c r="A65" s="74" t="s">
         <v>2</v>
       </c>
-      <c r="B65" s="54"/>
-      <c r="C65" s="54"/>
-      <c r="D65" s="54"/>
-      <c r="E65" s="54"/>
-      <c r="F65" s="54"/>
-      <c r="G65" s="55"/>
+      <c r="B65" s="75"/>
+      <c r="C65" s="75"/>
+      <c r="D65" s="75"/>
+      <c r="E65" s="75"/>
+      <c r="F65" s="75"/>
+      <c r="G65" s="76"/>
     </row>
     <row r="66" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A66" s="83" t="s">
+      <c r="A66" s="77" t="s">
         <v>3</v>
       </c>
-      <c r="B66" s="61"/>
-      <c r="C66" s="61"/>
-      <c r="D66" s="61"/>
-      <c r="E66" s="61"/>
-      <c r="F66" s="61"/>
-      <c r="G66" s="62"/>
+      <c r="B66" s="64"/>
+      <c r="C66" s="64"/>
+      <c r="D66" s="64"/>
+      <c r="E66" s="64"/>
+      <c r="F66" s="64"/>
+      <c r="G66" s="65"/>
     </row>
     <row r="67" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A67" s="75"/>
+      <c r="A67" s="61"/>
       <c r="B67" s="57"/>
       <c r="C67" s="57"/>
       <c r="D67" s="57"/>
       <c r="E67" s="57"/>
       <c r="F67" s="57"/>
-      <c r="G67" s="64"/>
+      <c r="G67" s="58"/>
     </row>
     <row r="68" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A68" s="68"/>
-      <c r="B68" s="69"/>
-      <c r="C68" s="69"/>
-      <c r="D68" s="69"/>
-      <c r="E68" s="69"/>
-      <c r="F68" s="69"/>
-      <c r="G68" s="70"/>
+      <c r="A68" s="60"/>
+      <c r="B68" s="54"/>
+      <c r="C68" s="54"/>
+      <c r="D68" s="54"/>
+      <c r="E68" s="54"/>
+      <c r="F68" s="54"/>
+      <c r="G68" s="55"/>
     </row>
     <row r="69" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A69" s="84" t="s">
+      <c r="A69" s="53" t="s">
         <v>4</v>
       </c>
-      <c r="B69" s="69"/>
-      <c r="C69" s="69"/>
-      <c r="D69" s="69"/>
-      <c r="E69" s="69"/>
-      <c r="F69" s="69"/>
-      <c r="G69" s="70"/>
+      <c r="B69" s="54"/>
+      <c r="C69" s="54"/>
+      <c r="D69" s="54"/>
+      <c r="E69" s="54"/>
+      <c r="F69" s="54"/>
+      <c r="G69" s="55"/>
     </row>
     <row r="70" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A70" s="85"/>
+      <c r="A70" s="56"/>
       <c r="B70" s="57"/>
       <c r="C70" s="57"/>
       <c r="D70" s="57"/>
       <c r="E70" s="57"/>
       <c r="F70" s="57"/>
-      <c r="G70" s="64"/>
+      <c r="G70" s="58"/>
     </row>
     <row r="71" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A71" s="65"/>
+      <c r="A71" s="59"/>
       <c r="B71" s="57"/>
       <c r="C71" s="57"/>
       <c r="D71" s="57"/>
       <c r="E71" s="57"/>
       <c r="F71" s="57"/>
-      <c r="G71" s="64"/>
+      <c r="G71" s="58"/>
     </row>
     <row r="72" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A72" s="65"/>
+      <c r="A72" s="59"/>
       <c r="B72" s="57"/>
       <c r="C72" s="57"/>
       <c r="D72" s="57"/>
       <c r="E72" s="57"/>
       <c r="F72" s="57"/>
-      <c r="G72" s="64"/>
+      <c r="G72" s="58"/>
     </row>
     <row r="73" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A73" s="68"/>
-      <c r="B73" s="69"/>
-      <c r="C73" s="69"/>
-      <c r="D73" s="69"/>
-      <c r="E73" s="69"/>
-      <c r="F73" s="69"/>
-      <c r="G73" s="70"/>
+      <c r="A73" s="60"/>
+      <c r="B73" s="54"/>
+      <c r="C73" s="54"/>
+      <c r="D73" s="54"/>
+      <c r="E73" s="54"/>
+      <c r="F73" s="54"/>
+      <c r="G73" s="55"/>
     </row>
     <row r="74" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A74" s="84" t="s">
+      <c r="A74" s="53" t="s">
         <v>5</v>
       </c>
-      <c r="B74" s="69"/>
-      <c r="C74" s="69"/>
-      <c r="D74" s="69"/>
-      <c r="E74" s="69"/>
-      <c r="F74" s="69"/>
-      <c r="G74" s="70"/>
+      <c r="B74" s="54"/>
+      <c r="C74" s="54"/>
+      <c r="D74" s="54"/>
+      <c r="E74" s="54"/>
+      <c r="F74" s="54"/>
+      <c r="G74" s="55"/>
     </row>
     <row r="75" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A75" s="75"/>
+      <c r="A75" s="61"/>
       <c r="B75" s="57"/>
       <c r="C75" s="57"/>
       <c r="D75" s="57"/>
       <c r="E75" s="57"/>
       <c r="F75" s="57"/>
-      <c r="G75" s="64"/>
+      <c r="G75" s="58"/>
     </row>
     <row r="76" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A76" s="68"/>
-      <c r="B76" s="69"/>
-      <c r="C76" s="69"/>
-      <c r="D76" s="69"/>
-      <c r="E76" s="69"/>
-      <c r="F76" s="69"/>
-      <c r="G76" s="70"/>
+      <c r="A76" s="60"/>
+      <c r="B76" s="54"/>
+      <c r="C76" s="54"/>
+      <c r="D76" s="54"/>
+      <c r="E76" s="54"/>
+      <c r="F76" s="54"/>
+      <c r="G76" s="55"/>
     </row>
     <row r="77" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A77" s="2"/>
@@ -2659,21 +2807,34 @@
       <c r="G78" s="46"/>
     </row>
     <row r="79" spans="1:7" ht="177.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A79" s="86"/>
-      <c r="B79" s="69"/>
-      <c r="C79" s="69"/>
-      <c r="D79" s="69"/>
-      <c r="E79" s="69"/>
-      <c r="F79" s="69"/>
-      <c r="G79" s="69"/>
+      <c r="A79" s="62"/>
+      <c r="B79" s="54"/>
+      <c r="C79" s="54"/>
+      <c r="D79" s="54"/>
+      <c r="E79" s="54"/>
+      <c r="F79" s="54"/>
+      <c r="G79" s="54"/>
     </row>
   </sheetData>
   <mergeCells count="35">
-    <mergeCell ref="A69:G69"/>
-    <mergeCell ref="A70:G73"/>
-    <mergeCell ref="A74:G74"/>
-    <mergeCell ref="A75:G76"/>
-    <mergeCell ref="A79:G79"/>
+    <mergeCell ref="A8:G8"/>
+    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A2:G2"/>
+    <mergeCell ref="A4:G4"/>
+    <mergeCell ref="A5:G5"/>
+    <mergeCell ref="A6:G7"/>
+    <mergeCell ref="A24:F24"/>
+    <mergeCell ref="A9:G12"/>
+    <mergeCell ref="A13:G13"/>
+    <mergeCell ref="A14:G15"/>
+    <mergeCell ref="A17:G17"/>
+    <mergeCell ref="A18:D18"/>
+    <mergeCell ref="E18:G18"/>
+    <mergeCell ref="A19:D19"/>
+    <mergeCell ref="E19:G19"/>
+    <mergeCell ref="A22:G22"/>
+    <mergeCell ref="A23:D23"/>
+    <mergeCell ref="E23:F23"/>
     <mergeCell ref="A67:G68"/>
     <mergeCell ref="A25:D25"/>
     <mergeCell ref="E25:F25"/>
@@ -2686,30 +2847,18 @@
     <mergeCell ref="A63:G63"/>
     <mergeCell ref="A65:G65"/>
     <mergeCell ref="A66:G66"/>
-    <mergeCell ref="A24:F24"/>
-    <mergeCell ref="A9:G12"/>
-    <mergeCell ref="A13:G13"/>
-    <mergeCell ref="A14:G15"/>
-    <mergeCell ref="A17:G17"/>
-    <mergeCell ref="A18:D18"/>
-    <mergeCell ref="E18:G18"/>
-    <mergeCell ref="A19:D19"/>
-    <mergeCell ref="E19:G19"/>
-    <mergeCell ref="A22:G22"/>
-    <mergeCell ref="A23:D23"/>
-    <mergeCell ref="E23:F23"/>
-    <mergeCell ref="A8:G8"/>
-    <mergeCell ref="A1:G1"/>
-    <mergeCell ref="A2:G2"/>
-    <mergeCell ref="A4:G4"/>
-    <mergeCell ref="A5:G5"/>
-    <mergeCell ref="A6:G7"/>
+    <mergeCell ref="A69:G69"/>
+    <mergeCell ref="A70:G73"/>
+    <mergeCell ref="A74:G74"/>
+    <mergeCell ref="A75:G76"/>
+    <mergeCell ref="A79:G79"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup scale="38" orientation="portrait" horizontalDpi="360" verticalDpi="360" r:id="rId1"/>
   <rowBreaks count="1" manualBreakCount="1">
     <brk id="36" max="16383" man="1"/>
   </rowBreaks>
+  <drawing r:id="rId2"/>
 </worksheet>
 </file>
 
@@ -2737,7 +2886,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:16" ht="25.8" x14ac:dyDescent="0.5">
-      <c r="A1" s="56" t="s">
+      <c r="A1" s="72" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="57"/>
@@ -2757,7 +2906,7 @@
       <c r="P1" s="57"/>
     </row>
     <row r="2" spans="1:16" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="58" t="s">
+      <c r="A2" s="73" t="s">
         <v>1</v>
       </c>
       <c r="B2" s="57"/>
@@ -2795,47 +2944,47 @@
       <c r="P3" s="2"/>
     </row>
     <row r="4" spans="1:16" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="88" t="s">
+      <c r="A4" s="101" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="54"/>
-      <c r="C4" s="54"/>
-      <c r="D4" s="54"/>
-      <c r="E4" s="54"/>
-      <c r="F4" s="54"/>
-      <c r="G4" s="54"/>
-      <c r="H4" s="54"/>
-      <c r="I4" s="54"/>
-      <c r="J4" s="54"/>
-      <c r="K4" s="54"/>
-      <c r="L4" s="54"/>
-      <c r="M4" s="54"/>
-      <c r="N4" s="54"/>
-      <c r="O4" s="54"/>
-      <c r="P4" s="55"/>
+      <c r="B4" s="75"/>
+      <c r="C4" s="75"/>
+      <c r="D4" s="75"/>
+      <c r="E4" s="75"/>
+      <c r="F4" s="75"/>
+      <c r="G4" s="75"/>
+      <c r="H4" s="75"/>
+      <c r="I4" s="75"/>
+      <c r="J4" s="75"/>
+      <c r="K4" s="75"/>
+      <c r="L4" s="75"/>
+      <c r="M4" s="75"/>
+      <c r="N4" s="75"/>
+      <c r="O4" s="75"/>
+      <c r="P4" s="76"/>
     </row>
     <row r="5" spans="1:16" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="87" t="s">
+      <c r="A5" s="98" t="s">
         <v>3</v>
       </c>
-      <c r="B5" s="54"/>
-      <c r="C5" s="54"/>
-      <c r="D5" s="54"/>
-      <c r="E5" s="54"/>
-      <c r="F5" s="54"/>
-      <c r="G5" s="54"/>
-      <c r="H5" s="54"/>
-      <c r="I5" s="54"/>
-      <c r="J5" s="54"/>
-      <c r="K5" s="54"/>
-      <c r="L5" s="54"/>
-      <c r="M5" s="54"/>
-      <c r="N5" s="54"/>
-      <c r="O5" s="54"/>
-      <c r="P5" s="55"/>
+      <c r="B5" s="75"/>
+      <c r="C5" s="75"/>
+      <c r="D5" s="75"/>
+      <c r="E5" s="75"/>
+      <c r="F5" s="75"/>
+      <c r="G5" s="75"/>
+      <c r="H5" s="75"/>
+      <c r="I5" s="75"/>
+      <c r="J5" s="75"/>
+      <c r="K5" s="75"/>
+      <c r="L5" s="75"/>
+      <c r="M5" s="75"/>
+      <c r="N5" s="75"/>
+      <c r="O5" s="75"/>
+      <c r="P5" s="76"/>
     </row>
     <row r="6" spans="1:16" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A6" s="75"/>
+      <c r="A6" s="61"/>
       <c r="B6" s="57"/>
       <c r="C6" s="57"/>
       <c r="D6" s="57"/>
@@ -2850,30 +2999,30 @@
       <c r="M6" s="57"/>
       <c r="N6" s="57"/>
       <c r="O6" s="57"/>
-      <c r="P6" s="64"/>
+      <c r="P6" s="58"/>
     </row>
     <row r="7" spans="1:16" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="87" t="s">
+      <c r="A7" s="98" t="s">
         <v>121</v>
       </c>
-      <c r="B7" s="54"/>
-      <c r="C7" s="54"/>
-      <c r="D7" s="54"/>
-      <c r="E7" s="54"/>
-      <c r="F7" s="54"/>
-      <c r="G7" s="54"/>
-      <c r="H7" s="54"/>
-      <c r="I7" s="54"/>
-      <c r="J7" s="54"/>
-      <c r="K7" s="54"/>
-      <c r="L7" s="54"/>
-      <c r="M7" s="54"/>
-      <c r="N7" s="54"/>
-      <c r="O7" s="54"/>
-      <c r="P7" s="55"/>
+      <c r="B7" s="75"/>
+      <c r="C7" s="75"/>
+      <c r="D7" s="75"/>
+      <c r="E7" s="75"/>
+      <c r="F7" s="75"/>
+      <c r="G7" s="75"/>
+      <c r="H7" s="75"/>
+      <c r="I7" s="75"/>
+      <c r="J7" s="75"/>
+      <c r="K7" s="75"/>
+      <c r="L7" s="75"/>
+      <c r="M7" s="75"/>
+      <c r="N7" s="75"/>
+      <c r="O7" s="75"/>
+      <c r="P7" s="76"/>
     </row>
     <row r="8" spans="1:16" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A8" s="85"/>
+      <c r="A8" s="56"/>
       <c r="B8" s="57"/>
       <c r="C8" s="57"/>
       <c r="D8" s="57"/>
@@ -2888,45 +3037,45 @@
       <c r="M8" s="57"/>
       <c r="N8" s="57"/>
       <c r="O8" s="57"/>
-      <c r="P8" s="64"/>
+      <c r="P8" s="58"/>
     </row>
     <row r="9" spans="1:16" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="87" t="s">
+      <c r="A9" s="98" t="s">
         <v>5</v>
       </c>
-      <c r="B9" s="54"/>
-      <c r="C9" s="54"/>
-      <c r="D9" s="54"/>
-      <c r="E9" s="54"/>
-      <c r="F9" s="54"/>
-      <c r="G9" s="54"/>
-      <c r="H9" s="54"/>
-      <c r="I9" s="54"/>
-      <c r="J9" s="54"/>
-      <c r="K9" s="54"/>
-      <c r="L9" s="54"/>
-      <c r="M9" s="54"/>
-      <c r="N9" s="54"/>
-      <c r="O9" s="54"/>
-      <c r="P9" s="55"/>
+      <c r="B9" s="75"/>
+      <c r="C9" s="75"/>
+      <c r="D9" s="75"/>
+      <c r="E9" s="75"/>
+      <c r="F9" s="75"/>
+      <c r="G9" s="75"/>
+      <c r="H9" s="75"/>
+      <c r="I9" s="75"/>
+      <c r="J9" s="75"/>
+      <c r="K9" s="75"/>
+      <c r="L9" s="75"/>
+      <c r="M9" s="75"/>
+      <c r="N9" s="75"/>
+      <c r="O9" s="75"/>
+      <c r="P9" s="76"/>
     </row>
     <row r="10" spans="1:16" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A10" s="89"/>
-      <c r="B10" s="69"/>
-      <c r="C10" s="69"/>
-      <c r="D10" s="69"/>
-      <c r="E10" s="69"/>
-      <c r="F10" s="69"/>
-      <c r="G10" s="69"/>
-      <c r="H10" s="69"/>
-      <c r="I10" s="69"/>
-      <c r="J10" s="69"/>
-      <c r="K10" s="69"/>
-      <c r="L10" s="69"/>
-      <c r="M10" s="69"/>
-      <c r="N10" s="69"/>
-      <c r="O10" s="69"/>
-      <c r="P10" s="70"/>
+      <c r="A10" s="99"/>
+      <c r="B10" s="54"/>
+      <c r="C10" s="54"/>
+      <c r="D10" s="54"/>
+      <c r="E10" s="54"/>
+      <c r="F10" s="54"/>
+      <c r="G10" s="54"/>
+      <c r="H10" s="54"/>
+      <c r="I10" s="54"/>
+      <c r="J10" s="54"/>
+      <c r="K10" s="54"/>
+      <c r="L10" s="54"/>
+      <c r="M10" s="54"/>
+      <c r="N10" s="54"/>
+      <c r="O10" s="54"/>
+      <c r="P10" s="55"/>
     </row>
     <row r="11" spans="1:16" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="2"/>
@@ -2947,68 +3096,68 @@
       <c r="P11" s="2"/>
     </row>
     <row r="12" spans="1:16" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="90" t="s">
+      <c r="A12" s="100" t="s">
         <v>6</v>
       </c>
-      <c r="B12" s="61"/>
-      <c r="C12" s="61"/>
-      <c r="D12" s="61"/>
-      <c r="E12" s="61"/>
-      <c r="F12" s="61"/>
-      <c r="G12" s="61"/>
-      <c r="H12" s="61"/>
-      <c r="I12" s="61"/>
-      <c r="J12" s="61"/>
-      <c r="K12" s="61"/>
-      <c r="L12" s="61"/>
-      <c r="M12" s="61"/>
-      <c r="N12" s="61"/>
-      <c r="O12" s="61"/>
-      <c r="P12" s="62"/>
+      <c r="B12" s="64"/>
+      <c r="C12" s="64"/>
+      <c r="D12" s="64"/>
+      <c r="E12" s="64"/>
+      <c r="F12" s="64"/>
+      <c r="G12" s="64"/>
+      <c r="H12" s="64"/>
+      <c r="I12" s="64"/>
+      <c r="J12" s="64"/>
+      <c r="K12" s="64"/>
+      <c r="L12" s="64"/>
+      <c r="M12" s="64"/>
+      <c r="N12" s="64"/>
+      <c r="O12" s="64"/>
+      <c r="P12" s="65"/>
     </row>
     <row r="13" spans="1:16" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="91">
+      <c r="A13" s="95">
         <v>1</v>
       </c>
-      <c r="B13" s="69"/>
-      <c r="C13" s="69"/>
-      <c r="D13" s="69"/>
-      <c r="E13" s="69"/>
-      <c r="F13" s="69"/>
-      <c r="G13" s="70"/>
-      <c r="H13" s="92">
+      <c r="B13" s="54"/>
+      <c r="C13" s="54"/>
+      <c r="D13" s="54"/>
+      <c r="E13" s="54"/>
+      <c r="F13" s="54"/>
+      <c r="G13" s="55"/>
+      <c r="H13" s="96">
         <v>3</v>
       </c>
-      <c r="I13" s="69"/>
-      <c r="J13" s="69"/>
-      <c r="K13" s="69"/>
-      <c r="L13" s="69"/>
-      <c r="M13" s="69"/>
-      <c r="N13" s="69"/>
-      <c r="O13" s="69"/>
-      <c r="P13" s="70"/>
+      <c r="I13" s="54"/>
+      <c r="J13" s="54"/>
+      <c r="K13" s="54"/>
+      <c r="L13" s="54"/>
+      <c r="M13" s="54"/>
+      <c r="N13" s="54"/>
+      <c r="O13" s="54"/>
+      <c r="P13" s="55"/>
     </row>
     <row r="14" spans="1:16" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="91">
+      <c r="A14" s="95">
         <v>2</v>
       </c>
-      <c r="B14" s="69"/>
-      <c r="C14" s="69"/>
-      <c r="D14" s="69"/>
-      <c r="E14" s="69"/>
-      <c r="F14" s="69"/>
-      <c r="G14" s="70"/>
-      <c r="H14" s="92">
+      <c r="B14" s="54"/>
+      <c r="C14" s="54"/>
+      <c r="D14" s="54"/>
+      <c r="E14" s="54"/>
+      <c r="F14" s="54"/>
+      <c r="G14" s="55"/>
+      <c r="H14" s="96">
         <v>4</v>
       </c>
-      <c r="I14" s="69"/>
-      <c r="J14" s="69"/>
-      <c r="K14" s="69"/>
-      <c r="L14" s="69"/>
-      <c r="M14" s="69"/>
-      <c r="N14" s="69"/>
-      <c r="O14" s="69"/>
-      <c r="P14" s="70"/>
+      <c r="I14" s="54"/>
+      <c r="J14" s="54"/>
+      <c r="K14" s="54"/>
+      <c r="L14" s="54"/>
+      <c r="M14" s="54"/>
+      <c r="N14" s="54"/>
+      <c r="O14" s="54"/>
+      <c r="P14" s="55"/>
     </row>
     <row r="15" spans="1:16" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="47"/>
@@ -3065,66 +3214,66 @@
       <c r="F17" s="49" t="s">
         <v>20</v>
       </c>
-      <c r="G17" s="93" t="s">
+      <c r="G17" s="97" t="s">
         <v>122</v>
       </c>
-      <c r="H17" s="61"/>
-      <c r="I17" s="61"/>
-      <c r="J17" s="61"/>
-      <c r="K17" s="61"/>
-      <c r="L17" s="61"/>
-      <c r="M17" s="61"/>
-      <c r="N17" s="61"/>
-      <c r="O17" s="61"/>
-      <c r="P17" s="62"/>
+      <c r="H17" s="64"/>
+      <c r="I17" s="64"/>
+      <c r="J17" s="64"/>
+      <c r="K17" s="64"/>
+      <c r="L17" s="64"/>
+      <c r="M17" s="64"/>
+      <c r="N17" s="64"/>
+      <c r="O17" s="64"/>
+      <c r="P17" s="65"/>
     </row>
     <row r="18" spans="1:16" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="94" t="s">
         <v>123</v>
       </c>
-      <c r="B18" s="96" t="s">
+      <c r="B18" s="91" t="s">
         <v>124</v>
       </c>
-      <c r="C18" s="96" t="s">
+      <c r="C18" s="91" t="s">
         <v>125</v>
       </c>
-      <c r="D18" s="96" t="s">
+      <c r="D18" s="91" t="s">
         <v>126</v>
       </c>
-      <c r="E18" s="96" t="s">
+      <c r="E18" s="91" t="s">
         <v>127</v>
       </c>
-      <c r="F18" s="96" t="s">
+      <c r="F18" s="91" t="s">
         <v>128</v>
       </c>
-      <c r="G18" s="97">
+      <c r="G18" s="93">
         <v>1</v>
       </c>
-      <c r="H18" s="62"/>
-      <c r="I18" s="97">
+      <c r="H18" s="65"/>
+      <c r="I18" s="93">
         <v>2</v>
       </c>
-      <c r="J18" s="62"/>
-      <c r="K18" s="97">
+      <c r="J18" s="65"/>
+      <c r="K18" s="93">
         <v>3</v>
       </c>
-      <c r="L18" s="62"/>
-      <c r="M18" s="97">
+      <c r="L18" s="65"/>
+      <c r="M18" s="93">
         <v>4</v>
       </c>
-      <c r="N18" s="62"/>
-      <c r="O18" s="97">
+      <c r="N18" s="65"/>
+      <c r="O18" s="93">
         <v>5</v>
       </c>
-      <c r="P18" s="62"/>
+      <c r="P18" s="65"/>
     </row>
     <row r="19" spans="1:16" ht="33.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A19" s="95"/>
-      <c r="B19" s="95"/>
-      <c r="C19" s="95"/>
-      <c r="D19" s="95"/>
-      <c r="E19" s="95"/>
-      <c r="F19" s="95"/>
+      <c r="A19" s="92"/>
+      <c r="B19" s="92"/>
+      <c r="C19" s="92"/>
+      <c r="D19" s="92"/>
+      <c r="E19" s="92"/>
+      <c r="F19" s="92"/>
       <c r="G19" s="50"/>
       <c r="H19" s="51">
         <f>G19*8</f>
@@ -3155,49 +3304,49 @@
       <c r="A20" s="94" t="s">
         <v>129</v>
       </c>
-      <c r="B20" s="96" t="s">
+      <c r="B20" s="91" t="s">
         <v>130</v>
       </c>
-      <c r="C20" s="96" t="s">
+      <c r="C20" s="91" t="s">
         <v>131</v>
       </c>
-      <c r="D20" s="96" t="s">
+      <c r="D20" s="91" t="s">
         <v>132</v>
       </c>
-      <c r="E20" s="96" t="s">
+      <c r="E20" s="91" t="s">
         <v>133</v>
       </c>
-      <c r="F20" s="96" t="s">
+      <c r="F20" s="91" t="s">
         <v>134</v>
       </c>
-      <c r="G20" s="97">
+      <c r="G20" s="93">
         <v>1</v>
       </c>
-      <c r="H20" s="62"/>
-      <c r="I20" s="97">
+      <c r="H20" s="65"/>
+      <c r="I20" s="93">
         <v>2</v>
       </c>
-      <c r="J20" s="62"/>
-      <c r="K20" s="97">
+      <c r="J20" s="65"/>
+      <c r="K20" s="93">
         <v>3</v>
       </c>
-      <c r="L20" s="62"/>
-      <c r="M20" s="97">
+      <c r="L20" s="65"/>
+      <c r="M20" s="93">
         <v>4</v>
       </c>
-      <c r="N20" s="62"/>
-      <c r="O20" s="97">
+      <c r="N20" s="65"/>
+      <c r="O20" s="93">
         <v>5</v>
       </c>
-      <c r="P20" s="62"/>
+      <c r="P20" s="65"/>
     </row>
     <row r="21" spans="1:16" ht="44.4" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A21" s="95"/>
-      <c r="B21" s="95"/>
-      <c r="C21" s="95"/>
-      <c r="D21" s="95"/>
-      <c r="E21" s="95"/>
-      <c r="F21" s="95"/>
+      <c r="A21" s="92"/>
+      <c r="B21" s="92"/>
+      <c r="C21" s="92"/>
+      <c r="D21" s="92"/>
+      <c r="E21" s="92"/>
+      <c r="F21" s="92"/>
       <c r="G21" s="50"/>
       <c r="H21" s="51">
         <f>G21*6</f>
@@ -3228,49 +3377,49 @@
       <c r="A22" s="94" t="s">
         <v>135</v>
       </c>
-      <c r="B22" s="96" t="s">
+      <c r="B22" s="91" t="s">
         <v>136</v>
       </c>
-      <c r="C22" s="96" t="s">
+      <c r="C22" s="91" t="s">
         <v>137</v>
       </c>
-      <c r="D22" s="96" t="s">
+      <c r="D22" s="91" t="s">
         <v>138</v>
       </c>
-      <c r="E22" s="96" t="s">
+      <c r="E22" s="91" t="s">
         <v>139</v>
       </c>
-      <c r="F22" s="96" t="s">
+      <c r="F22" s="91" t="s">
         <v>140</v>
       </c>
-      <c r="G22" s="97">
+      <c r="G22" s="93">
         <v>1</v>
       </c>
-      <c r="H22" s="62"/>
-      <c r="I22" s="97">
+      <c r="H22" s="65"/>
+      <c r="I22" s="93">
         <v>2</v>
       </c>
-      <c r="J22" s="62"/>
-      <c r="K22" s="97">
+      <c r="J22" s="65"/>
+      <c r="K22" s="93">
         <v>3</v>
       </c>
-      <c r="L22" s="62"/>
-      <c r="M22" s="97">
+      <c r="L22" s="65"/>
+      <c r="M22" s="93">
         <v>4</v>
       </c>
-      <c r="N22" s="62"/>
-      <c r="O22" s="97">
+      <c r="N22" s="65"/>
+      <c r="O22" s="93">
         <v>5</v>
       </c>
-      <c r="P22" s="62"/>
+      <c r="P22" s="65"/>
     </row>
     <row r="23" spans="1:16" ht="28.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A23" s="95"/>
-      <c r="B23" s="95"/>
-      <c r="C23" s="95"/>
-      <c r="D23" s="95"/>
-      <c r="E23" s="95"/>
-      <c r="F23" s="95"/>
+      <c r="A23" s="92"/>
+      <c r="B23" s="92"/>
+      <c r="C23" s="92"/>
+      <c r="D23" s="92"/>
+      <c r="E23" s="92"/>
+      <c r="F23" s="92"/>
       <c r="G23" s="50"/>
       <c r="H23" s="52">
         <f>G23*2</f>
@@ -3301,45 +3450,45 @@
       <c r="A24" s="94" t="s">
         <v>141</v>
       </c>
-      <c r="B24" s="96" t="s">
+      <c r="B24" s="91" t="s">
         <v>142</v>
       </c>
-      <c r="C24" s="96" t="s">
+      <c r="C24" s="91" t="s">
         <v>143</v>
       </c>
-      <c r="D24" s="96" t="s">
+      <c r="D24" s="91" t="s">
         <v>144</v>
       </c>
-      <c r="E24" s="96" t="s">
+      <c r="E24" s="91" t="s">
         <v>145</v>
       </c>
-      <c r="F24" s="96" t="s">
+      <c r="F24" s="91" t="s">
         <v>146</v>
       </c>
-      <c r="G24" s="97">
+      <c r="G24" s="93">
         <v>1</v>
       </c>
-      <c r="H24" s="62"/>
-      <c r="I24" s="97">
+      <c r="H24" s="65"/>
+      <c r="I24" s="93">
         <v>2</v>
       </c>
-      <c r="J24" s="62"/>
-      <c r="K24" s="97"/>
-      <c r="L24" s="62"/>
-      <c r="M24" s="97"/>
-      <c r="N24" s="62"/>
-      <c r="O24" s="97">
+      <c r="J24" s="65"/>
+      <c r="K24" s="93"/>
+      <c r="L24" s="65"/>
+      <c r="M24" s="93"/>
+      <c r="N24" s="65"/>
+      <c r="O24" s="93">
         <v>5</v>
       </c>
-      <c r="P24" s="62"/>
+      <c r="P24" s="65"/>
     </row>
     <row r="25" spans="1:16" ht="28.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A25" s="95"/>
-      <c r="B25" s="95"/>
-      <c r="C25" s="95"/>
-      <c r="D25" s="95"/>
-      <c r="E25" s="95"/>
-      <c r="F25" s="95"/>
+      <c r="A25" s="92"/>
+      <c r="B25" s="92"/>
+      <c r="C25" s="92"/>
+      <c r="D25" s="92"/>
+      <c r="E25" s="92"/>
+      <c r="F25" s="92"/>
       <c r="G25" s="50"/>
       <c r="H25" s="52">
         <f>G25*2</f>
@@ -3370,49 +3519,49 @@
       <c r="A26" s="94" t="s">
         <v>147</v>
       </c>
-      <c r="B26" s="96" t="s">
+      <c r="B26" s="91" t="s">
         <v>148</v>
       </c>
-      <c r="C26" s="96" t="s">
+      <c r="C26" s="91" t="s">
         <v>149</v>
       </c>
-      <c r="D26" s="96" t="s">
+      <c r="D26" s="91" t="s">
         <v>150</v>
       </c>
-      <c r="E26" s="96" t="s">
+      <c r="E26" s="91" t="s">
         <v>151</v>
       </c>
-      <c r="F26" s="96" t="s">
+      <c r="F26" s="91" t="s">
         <v>152</v>
       </c>
-      <c r="G26" s="97">
+      <c r="G26" s="93">
         <v>1</v>
       </c>
-      <c r="H26" s="62"/>
-      <c r="I26" s="97">
+      <c r="H26" s="65"/>
+      <c r="I26" s="93">
         <v>2</v>
       </c>
-      <c r="J26" s="62"/>
-      <c r="K26" s="97">
+      <c r="J26" s="65"/>
+      <c r="K26" s="93">
         <v>3</v>
       </c>
-      <c r="L26" s="62"/>
-      <c r="M26" s="97">
+      <c r="L26" s="65"/>
+      <c r="M26" s="93">
         <v>4</v>
       </c>
-      <c r="N26" s="62"/>
-      <c r="O26" s="97">
+      <c r="N26" s="65"/>
+      <c r="O26" s="93">
         <v>5</v>
       </c>
-      <c r="P26" s="62"/>
+      <c r="P26" s="65"/>
     </row>
     <row r="27" spans="1:16" ht="28.8" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A27" s="95"/>
-      <c r="B27" s="95"/>
-      <c r="C27" s="95"/>
-      <c r="D27" s="95"/>
-      <c r="E27" s="95"/>
-      <c r="F27" s="95"/>
+      <c r="A27" s="92"/>
+      <c r="B27" s="92"/>
+      <c r="C27" s="92"/>
+      <c r="D27" s="92"/>
+      <c r="E27" s="92"/>
+      <c r="F27" s="92"/>
       <c r="G27" s="50"/>
       <c r="H27" s="52">
         <f>G27*2</f>
@@ -3440,39 +3589,39 @@
       </c>
     </row>
     <row r="28" spans="1:16" ht="33" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A28" s="101" t="s">
+      <c r="A28" s="89" t="s">
         <v>153</v>
       </c>
-      <c r="B28" s="61"/>
-      <c r="C28" s="61"/>
-      <c r="D28" s="61"/>
-      <c r="E28" s="61"/>
-      <c r="F28" s="62"/>
-      <c r="G28" s="98">
+      <c r="B28" s="64"/>
+      <c r="C28" s="64"/>
+      <c r="D28" s="64"/>
+      <c r="E28" s="64"/>
+      <c r="F28" s="65"/>
+      <c r="G28" s="90">
         <f>SUM(H19,H21,H23,H25,H27)</f>
         <v>0</v>
       </c>
-      <c r="H28" s="62"/>
-      <c r="I28" s="98">
+      <c r="H28" s="65"/>
+      <c r="I28" s="90">
         <f>SUM(J19,J21,J23,J25,J27)</f>
         <v>0</v>
       </c>
-      <c r="J28" s="62"/>
-      <c r="K28" s="98">
+      <c r="J28" s="65"/>
+      <c r="K28" s="90">
         <f>SUM(L19,L21,L23,L25,L27)</f>
         <v>0</v>
       </c>
-      <c r="L28" s="62"/>
-      <c r="M28" s="98">
+      <c r="L28" s="65"/>
+      <c r="M28" s="90">
         <f>SUM(N19,N21,N23,N25,N27)</f>
         <v>0</v>
       </c>
-      <c r="N28" s="62"/>
-      <c r="O28" s="98">
+      <c r="N28" s="65"/>
+      <c r="O28" s="90">
         <f>SUM(P19,P21,P23,P25,P27)</f>
         <v>0</v>
       </c>
-      <c r="P28" s="62"/>
+      <c r="P28" s="65"/>
     </row>
     <row r="29" spans="1:16" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A29" s="2"/>
@@ -3498,12 +3647,12 @@
       <c r="C30" s="2"/>
       <c r="D30" s="2"/>
       <c r="E30" s="2"/>
-      <c r="F30" s="99" t="s">
+      <c r="F30" s="87" t="s">
         <v>117</v>
       </c>
-      <c r="G30" s="69"/>
-      <c r="H30" s="69"/>
-      <c r="I30" s="69"/>
+      <c r="G30" s="54"/>
+      <c r="H30" s="54"/>
+      <c r="I30" s="54"/>
       <c r="J30" s="2"/>
       <c r="K30" s="2"/>
       <c r="L30" s="2"/>
@@ -3518,7 +3667,7 @@
       <c r="C31" s="2"/>
       <c r="D31" s="2"/>
       <c r="E31" s="2"/>
-      <c r="F31" s="100" t="s">
+      <c r="F31" s="88" t="s">
         <v>154</v>
       </c>
       <c r="G31" s="57"/>
@@ -7902,58 +8051,18 @@
     <row r="999" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
   </sheetData>
   <mergeCells count="78">
-    <mergeCell ref="F30:I30"/>
-    <mergeCell ref="F31:I31"/>
-    <mergeCell ref="A28:F28"/>
-    <mergeCell ref="G28:H28"/>
-    <mergeCell ref="I28:J28"/>
-    <mergeCell ref="F26:F27"/>
-    <mergeCell ref="G26:H26"/>
-    <mergeCell ref="I26:J26"/>
-    <mergeCell ref="K26:L26"/>
-    <mergeCell ref="M26:N26"/>
-    <mergeCell ref="M24:N24"/>
-    <mergeCell ref="O24:P24"/>
-    <mergeCell ref="K28:L28"/>
-    <mergeCell ref="M28:N28"/>
-    <mergeCell ref="O28:P28"/>
-    <mergeCell ref="O26:P26"/>
-    <mergeCell ref="A26:A27"/>
-    <mergeCell ref="B26:B27"/>
-    <mergeCell ref="C26:C27"/>
-    <mergeCell ref="D26:D27"/>
-    <mergeCell ref="E26:E27"/>
-    <mergeCell ref="A24:A25"/>
-    <mergeCell ref="B24:B25"/>
-    <mergeCell ref="C24:C25"/>
-    <mergeCell ref="D24:D25"/>
-    <mergeCell ref="E24:E25"/>
-    <mergeCell ref="F24:F25"/>
-    <mergeCell ref="F22:F23"/>
-    <mergeCell ref="G22:H22"/>
-    <mergeCell ref="I22:J22"/>
-    <mergeCell ref="K22:L22"/>
-    <mergeCell ref="G24:H24"/>
-    <mergeCell ref="I24:J24"/>
-    <mergeCell ref="K24:L24"/>
-    <mergeCell ref="M22:N22"/>
-    <mergeCell ref="O22:P22"/>
-    <mergeCell ref="G20:H20"/>
-    <mergeCell ref="I20:J20"/>
-    <mergeCell ref="K20:L20"/>
-    <mergeCell ref="M20:N20"/>
-    <mergeCell ref="O20:P20"/>
-    <mergeCell ref="F20:F21"/>
-    <mergeCell ref="A22:A23"/>
-    <mergeCell ref="B22:B23"/>
-    <mergeCell ref="C22:C23"/>
-    <mergeCell ref="D22:D23"/>
-    <mergeCell ref="E22:E23"/>
-    <mergeCell ref="A20:A21"/>
-    <mergeCell ref="B20:B21"/>
-    <mergeCell ref="C20:C21"/>
-    <mergeCell ref="D20:D21"/>
-    <mergeCell ref="E20:E21"/>
+    <mergeCell ref="A7:P7"/>
+    <mergeCell ref="A1:P1"/>
+    <mergeCell ref="A2:P2"/>
+    <mergeCell ref="A4:P4"/>
+    <mergeCell ref="A5:P5"/>
+    <mergeCell ref="A6:P6"/>
+    <mergeCell ref="A8:P8"/>
+    <mergeCell ref="A9:P9"/>
+    <mergeCell ref="A10:P10"/>
+    <mergeCell ref="A12:P12"/>
+    <mergeCell ref="A13:G13"/>
+    <mergeCell ref="H13:P13"/>
     <mergeCell ref="A14:G14"/>
     <mergeCell ref="H14:P14"/>
     <mergeCell ref="G17:P17"/>
@@ -7968,19 +8077,60 @@
     <mergeCell ref="K18:L18"/>
     <mergeCell ref="M18:N18"/>
     <mergeCell ref="O18:P18"/>
-    <mergeCell ref="A8:P8"/>
-    <mergeCell ref="A9:P9"/>
-    <mergeCell ref="A10:P10"/>
-    <mergeCell ref="A12:P12"/>
-    <mergeCell ref="A13:G13"/>
-    <mergeCell ref="H13:P13"/>
-    <mergeCell ref="A7:P7"/>
-    <mergeCell ref="A1:P1"/>
-    <mergeCell ref="A2:P2"/>
-    <mergeCell ref="A4:P4"/>
-    <mergeCell ref="A5:P5"/>
-    <mergeCell ref="A6:P6"/>
+    <mergeCell ref="F20:F21"/>
+    <mergeCell ref="A22:A23"/>
+    <mergeCell ref="B22:B23"/>
+    <mergeCell ref="C22:C23"/>
+    <mergeCell ref="D22:D23"/>
+    <mergeCell ref="E22:E23"/>
+    <mergeCell ref="A20:A21"/>
+    <mergeCell ref="B20:B21"/>
+    <mergeCell ref="C20:C21"/>
+    <mergeCell ref="D20:D21"/>
+    <mergeCell ref="E20:E21"/>
+    <mergeCell ref="M22:N22"/>
+    <mergeCell ref="O22:P22"/>
+    <mergeCell ref="G20:H20"/>
+    <mergeCell ref="I20:J20"/>
+    <mergeCell ref="K20:L20"/>
+    <mergeCell ref="M20:N20"/>
+    <mergeCell ref="O20:P20"/>
+    <mergeCell ref="F24:F25"/>
+    <mergeCell ref="F22:F23"/>
+    <mergeCell ref="G22:H22"/>
+    <mergeCell ref="I22:J22"/>
+    <mergeCell ref="K22:L22"/>
+    <mergeCell ref="G24:H24"/>
+    <mergeCell ref="I24:J24"/>
+    <mergeCell ref="K24:L24"/>
+    <mergeCell ref="A24:A25"/>
+    <mergeCell ref="B24:B25"/>
+    <mergeCell ref="C24:C25"/>
+    <mergeCell ref="D24:D25"/>
+    <mergeCell ref="E24:E25"/>
+    <mergeCell ref="A26:A27"/>
+    <mergeCell ref="B26:B27"/>
+    <mergeCell ref="C26:C27"/>
+    <mergeCell ref="D26:D27"/>
+    <mergeCell ref="E26:E27"/>
+    <mergeCell ref="M24:N24"/>
+    <mergeCell ref="O24:P24"/>
+    <mergeCell ref="K28:L28"/>
+    <mergeCell ref="M28:N28"/>
+    <mergeCell ref="O28:P28"/>
+    <mergeCell ref="O26:P26"/>
+    <mergeCell ref="F26:F27"/>
+    <mergeCell ref="G26:H26"/>
+    <mergeCell ref="I26:J26"/>
+    <mergeCell ref="K26:L26"/>
+    <mergeCell ref="M26:N26"/>
+    <mergeCell ref="F30:I30"/>
+    <mergeCell ref="F31:I31"/>
+    <mergeCell ref="A28:F28"/>
+    <mergeCell ref="G28:H28"/>
+    <mergeCell ref="I28:J28"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>